<commit_message>
Card Drop logic cleanup
</commit_message>
<xml_diff>
--- a/Assets/CardLibrary/CardLibrary.xlsx
+++ b/Assets/CardLibrary/CardLibrary.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Poet\Assets\CardLibrary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3A6BCA-8F34-4596-8283-D4CCD6B4876A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2A8AEE-FE03-4CC3-8014-49C1A59883A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="826" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FullLibrary" sheetId="1" r:id="rId1"/>
     <sheet name="Raw_Choice" sheetId="5" r:id="rId2"/>
-    <sheet name="ForgeLibrary_Universal" sheetId="6" r:id="rId3"/>
-    <sheet name="ForgeLibrary_Nature" sheetId="8" r:id="rId4"/>
-    <sheet name="ForgeLibrary_Politics" sheetId="9" r:id="rId5"/>
-    <sheet name="ForgeLibrary_Emotion" sheetId="7" r:id="rId6"/>
-    <sheet name="Node" sheetId="10" r:id="rId7"/>
+    <sheet name="EventCard_Choices" sheetId="12" r:id="rId3"/>
+    <sheet name="ForgeLibrary_Universal" sheetId="6" r:id="rId4"/>
+    <sheet name="ForgeLibrary_Nature" sheetId="8" r:id="rId5"/>
+    <sheet name="ForgeLibrary_Politics" sheetId="9" r:id="rId6"/>
+    <sheet name="ForgeLibrary_Emotion" sheetId="7" r:id="rId7"/>
     <sheet name="DailyMission" sheetId="11" r:id="rId8"/>
+    <sheet name="Node" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="239">
   <si>
     <t>Index</t>
   </si>
@@ -2662,6 +2663,40 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BEFD67-833C-4C4B-AEEA-212EA8D4541D}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:R18"/>
   <sheetFormatPr defaultColWidth="5.625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3077,7 +3112,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M29"/>
   <sheetFormatPr defaultColWidth="5.625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3186,7 +3221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="5.625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3234,7 +3269,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="5.625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3274,196 +3309,6 @@
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>131</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="14.875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3556,4 +3401,194 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="14.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>